<commit_message>
Organik ürün taşıma arabası adı tek: TR/EN/AR; tabela, etiket, plaka, talimat, formlar ve site güncellendi; organik formlarda başlık üç dilli
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6foNXTwf1dGzDjULYpfrk
</commit_message>
<xml_diff>
--- a/formlar/16. Organik Üretim/EMS.OR.FRM.21.01. Organik Hammadde Kabul ve TC Doğrulama Formu.xlsx
+++ b/formlar/16. Organik Üretim/EMS.OR.FRM.21.01. Organik Hammadde Kabul ve TC Doğrulama Formu.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -96,6 +96,12 @@
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -130,7 +136,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -262,11 +268,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -363,6 +397,11 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,6 +506,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -497,6 +539,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -822,23 +867,24 @@
       <c r="A1" s="25" t="n"/>
       <c r="B1" s="26" t="n"/>
       <c r="C1" s="27" t="n"/>
-      <c r="D1" s="28" t="inlineStr">
-        <is>
-          <t>ORGANIC RAW MATERIAL RECEIVING AND TC VERIFICATION FORM
+      <c r="D1" s="46" t="inlineStr">
+        <is>
+          <t>ORGANİK HAMMADDE KABUL VE TC DOĞRULAMA FORMU
+ORGANIC RAW MATERIAL RECEIVING AND TC VERIFICATION FORM
 نموذج استلام المواد الخام العضوية والتحقق من شهادة المعاملة</t>
         </is>
       </c>
-      <c r="E1" s="26" t="n"/>
-      <c r="F1" s="26" t="n"/>
-      <c r="G1" s="26" t="n"/>
-      <c r="H1" s="26" t="n"/>
-      <c r="I1" s="26" t="n"/>
-      <c r="J1" s="26" t="n"/>
-      <c r="K1" s="26" t="n"/>
-      <c r="L1" s="26" t="n"/>
-      <c r="M1" s="26" t="n"/>
-      <c r="N1" s="26" t="n"/>
-      <c r="O1" s="26" t="n"/>
+      <c r="E1" s="47" t="n"/>
+      <c r="F1" s="47" t="n"/>
+      <c r="G1" s="47" t="n"/>
+      <c r="H1" s="47" t="n"/>
+      <c r="I1" s="47" t="n"/>
+      <c r="J1" s="47" t="n"/>
+      <c r="K1" s="47" t="n"/>
+      <c r="L1" s="47" t="n"/>
+      <c r="M1" s="47" t="n"/>
+      <c r="N1" s="47" t="n"/>
+      <c r="O1" s="47" t="n"/>
       <c r="P1" s="26" t="n"/>
       <c r="Q1" s="26" t="n"/>
       <c r="R1" s="29" t="inlineStr">
@@ -846,7 +892,7 @@
           <t>DATE / التاريخ</t>
         </is>
       </c>
-      <c r="S1" s="30" t="n"/>
+      <c r="S1" s="48" t="n"/>
       <c r="T1" s="31" t="inlineStr">
         <is>
           <t>….../….../.…</t>
@@ -857,18 +903,6 @@
       <c r="A2" s="32" t="n"/>
       <c r="B2" s="33" t="n"/>
       <c r="C2" s="33" t="n"/>
-      <c r="D2" s="33" t="n"/>
-      <c r="E2" s="33" t="n"/>
-      <c r="F2" s="33" t="n"/>
-      <c r="G2" s="33" t="n"/>
-      <c r="H2" s="33" t="n"/>
-      <c r="I2" s="33" t="n"/>
-      <c r="J2" s="33" t="n"/>
-      <c r="K2" s="33" t="n"/>
-      <c r="L2" s="33" t="n"/>
-      <c r="M2" s="33" t="n"/>
-      <c r="N2" s="33" t="n"/>
-      <c r="O2" s="33" t="n"/>
       <c r="P2" s="33" t="n"/>
       <c r="Q2" s="33" t="n"/>
       <c r="R2" s="29" t="inlineStr">
@@ -876,7 +910,7 @@
           <t>FORM NUMBER / رقم النموذج</t>
         </is>
       </c>
-      <c r="S2" s="30" t="n"/>
+      <c r="S2" s="48" t="n"/>
       <c r="T2" s="34" t="inlineStr">
         <is>
           <t>EMS.OR.FRM.21.01</t>
@@ -887,18 +921,6 @@
       <c r="A3" s="32" t="n"/>
       <c r="B3" s="33" t="n"/>
       <c r="C3" s="33" t="n"/>
-      <c r="D3" s="33" t="n"/>
-      <c r="E3" s="33" t="n"/>
-      <c r="F3" s="33" t="n"/>
-      <c r="G3" s="33" t="n"/>
-      <c r="H3" s="33" t="n"/>
-      <c r="I3" s="33" t="n"/>
-      <c r="J3" s="33" t="n"/>
-      <c r="K3" s="33" t="n"/>
-      <c r="L3" s="33" t="n"/>
-      <c r="M3" s="33" t="n"/>
-      <c r="N3" s="33" t="n"/>
-      <c r="O3" s="33" t="n"/>
       <c r="P3" s="33" t="n"/>
       <c r="Q3" s="33" t="n"/>
       <c r="R3" s="29" t="inlineStr">
@@ -906,7 +928,7 @@
           <t>REVISION / المراجعة</t>
         </is>
       </c>
-      <c r="S3" s="30" t="n"/>
+      <c r="S3" s="48" t="n"/>
       <c r="T3" s="31" t="inlineStr">
         <is>
           <t>R00</t>
@@ -917,18 +939,6 @@
       <c r="A4" s="32" t="n"/>
       <c r="B4" s="33" t="n"/>
       <c r="C4" s="33" t="n"/>
-      <c r="D4" s="33" t="n"/>
-      <c r="E4" s="33" t="n"/>
-      <c r="F4" s="33" t="n"/>
-      <c r="G4" s="33" t="n"/>
-      <c r="H4" s="33" t="n"/>
-      <c r="I4" s="33" t="n"/>
-      <c r="J4" s="33" t="n"/>
-      <c r="K4" s="33" t="n"/>
-      <c r="L4" s="33" t="n"/>
-      <c r="M4" s="33" t="n"/>
-      <c r="N4" s="33" t="n"/>
-      <c r="O4" s="33" t="n"/>
       <c r="P4" s="33" t="n"/>
       <c r="Q4" s="33" t="n"/>
       <c r="R4" s="29" t="inlineStr">
@@ -936,14 +946,13 @@
           <t>PUBLIC. DATE / تاريخ النشر</t>
         </is>
       </c>
-      <c r="S4" s="30" t="n"/>
+      <c r="S4" s="48" t="n"/>
       <c r="T4" s="31" t="inlineStr">
         <is>
           <t>19.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
@@ -1049,7 +1058,6 @@
       <c r="S8" s="36" t="n"/>
       <c r="T8" s="37" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
@@ -1382,7 +1390,6 @@
       <c r="S21" s="17" t="n"/>
       <c r="T21" s="37" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="35" t="inlineStr">
         <is>
@@ -1741,7 +1748,6 @@
       </c>
       <c r="T31" s="37" t="n"/>
     </row>
-    <row r="32"/>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="35" t="inlineStr">
         <is>
@@ -1820,40 +1826,39 @@
       <c r="S36" s="41" t="n"/>
       <c r="T36" s="11" t="n"/>
     </row>
-    <row r="37"/>
     <row r="38" ht="26" customHeight="1">
       <c r="A38" s="42" t="inlineStr">
         <is>
           <t>Warehouse / المستودع</t>
         </is>
       </c>
-      <c r="B38" s="43" t="n"/>
-      <c r="C38" s="43" t="n"/>
-      <c r="D38" s="43" t="n"/>
-      <c r="E38" s="43" t="n"/>
-      <c r="F38" s="43" t="n"/>
-      <c r="G38" s="44" t="n"/>
+      <c r="B38" s="36" t="n"/>
+      <c r="C38" s="36" t="n"/>
+      <c r="D38" s="36" t="n"/>
+      <c r="E38" s="36" t="n"/>
+      <c r="F38" s="36" t="n"/>
+      <c r="G38" s="37" t="n"/>
       <c r="H38" s="42" t="inlineStr">
         <is>
           <t>OCS / GOTS Coordinator / منسق OCS / GOTS</t>
         </is>
       </c>
-      <c r="I38" s="43" t="n"/>
-      <c r="J38" s="43" t="n"/>
-      <c r="K38" s="43" t="n"/>
-      <c r="L38" s="43" t="n"/>
-      <c r="M38" s="43" t="n"/>
-      <c r="N38" s="44" t="n"/>
+      <c r="I38" s="36" t="n"/>
+      <c r="J38" s="36" t="n"/>
+      <c r="K38" s="36" t="n"/>
+      <c r="L38" s="36" t="n"/>
+      <c r="M38" s="36" t="n"/>
+      <c r="N38" s="37" t="n"/>
       <c r="O38" s="42" t="inlineStr">
         <is>
           <t>Quality / الجودة</t>
         </is>
       </c>
-      <c r="P38" s="43" t="n"/>
-      <c r="Q38" s="43" t="n"/>
-      <c r="R38" s="43" t="n"/>
-      <c r="S38" s="43" t="n"/>
-      <c r="T38" s="44" t="n"/>
+      <c r="P38" s="36" t="n"/>
+      <c r="Q38" s="36" t="n"/>
+      <c r="R38" s="36" t="n"/>
+      <c r="S38" s="36" t="n"/>
+      <c r="T38" s="37" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="23" t="inlineStr">
@@ -1919,32 +1924,31 @@
       <c r="S41" s="41" t="n"/>
       <c r="T41" s="11" t="n"/>
     </row>
-    <row r="42"/>
     <row r="43" ht="32" customHeight="1">
       <c r="A43" s="35" t="inlineStr">
         <is>
           <t>Retention: at least 5 years or per certification body / customer requirement. Any nonconformity opens a corrective action (DÖF). | الاحتفاظ: 5 سنوات على الأقل أو حسب متطلبات جهة الاعتماد / العميل. وتفتح أي حالة عدم مطابقة إجراءً تصحيحيًا (DÖF).</t>
         </is>
       </c>
-      <c r="B43" s="43" t="n"/>
-      <c r="C43" s="43" t="n"/>
-      <c r="D43" s="43" t="n"/>
-      <c r="E43" s="43" t="n"/>
-      <c r="F43" s="43" t="n"/>
-      <c r="G43" s="43" t="n"/>
-      <c r="H43" s="43" t="n"/>
-      <c r="I43" s="43" t="n"/>
-      <c r="J43" s="43" t="n"/>
-      <c r="K43" s="43" t="n"/>
-      <c r="L43" s="43" t="n"/>
-      <c r="M43" s="43" t="n"/>
-      <c r="N43" s="43" t="n"/>
-      <c r="O43" s="43" t="n"/>
-      <c r="P43" s="43" t="n"/>
-      <c r="Q43" s="43" t="n"/>
-      <c r="R43" s="43" t="n"/>
-      <c r="S43" s="43" t="n"/>
-      <c r="T43" s="44" t="n"/>
+      <c r="B43" s="36" t="n"/>
+      <c r="C43" s="36" t="n"/>
+      <c r="D43" s="36" t="n"/>
+      <c r="E43" s="36" t="n"/>
+      <c r="F43" s="36" t="n"/>
+      <c r="G43" s="36" t="n"/>
+      <c r="H43" s="36" t="n"/>
+      <c r="I43" s="36" t="n"/>
+      <c r="J43" s="36" t="n"/>
+      <c r="K43" s="36" t="n"/>
+      <c r="L43" s="36" t="n"/>
+      <c r="M43" s="36" t="n"/>
+      <c r="N43" s="36" t="n"/>
+      <c r="O43" s="36" t="n"/>
+      <c r="P43" s="36" t="n"/>
+      <c r="Q43" s="36" t="n"/>
+      <c r="R43" s="36" t="n"/>
+      <c r="S43" s="36" t="n"/>
+      <c r="T43" s="37" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="145">

</xml_diff>

<commit_message>
Organik ürün taşıma arabası adı tek: TR/EN/AR; tabela, etiket, plaka, talimat, formlar ve site güncellendi; organik formlarda başlık üç dilli (#465)
Claude-Session: https://claude.ai/code/session_01J6foNXTwf1dGzDjULYpfrk

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/formlar/16. Organik Üretim/EMS.OR.FRM.21.01. Organik Hammadde Kabul ve TC Doğrulama Formu.xlsx
+++ b/formlar/16. Organik Üretim/EMS.OR.FRM.21.01. Organik Hammadde Kabul ve TC Doğrulama Formu.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -96,6 +96,12 @@
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -130,7 +136,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -262,11 +268,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -363,6 +397,11 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,6 +506,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -497,6 +539,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -822,23 +867,24 @@
       <c r="A1" s="25" t="n"/>
       <c r="B1" s="26" t="n"/>
       <c r="C1" s="27" t="n"/>
-      <c r="D1" s="28" t="inlineStr">
-        <is>
-          <t>ORGANIC RAW MATERIAL RECEIVING AND TC VERIFICATION FORM
+      <c r="D1" s="46" t="inlineStr">
+        <is>
+          <t>ORGANİK HAMMADDE KABUL VE TC DOĞRULAMA FORMU
+ORGANIC RAW MATERIAL RECEIVING AND TC VERIFICATION FORM
 نموذج استلام المواد الخام العضوية والتحقق من شهادة المعاملة</t>
         </is>
       </c>
-      <c r="E1" s="26" t="n"/>
-      <c r="F1" s="26" t="n"/>
-      <c r="G1" s="26" t="n"/>
-      <c r="H1" s="26" t="n"/>
-      <c r="I1" s="26" t="n"/>
-      <c r="J1" s="26" t="n"/>
-      <c r="K1" s="26" t="n"/>
-      <c r="L1" s="26" t="n"/>
-      <c r="M1" s="26" t="n"/>
-      <c r="N1" s="26" t="n"/>
-      <c r="O1" s="26" t="n"/>
+      <c r="E1" s="47" t="n"/>
+      <c r="F1" s="47" t="n"/>
+      <c r="G1" s="47" t="n"/>
+      <c r="H1" s="47" t="n"/>
+      <c r="I1" s="47" t="n"/>
+      <c r="J1" s="47" t="n"/>
+      <c r="K1" s="47" t="n"/>
+      <c r="L1" s="47" t="n"/>
+      <c r="M1" s="47" t="n"/>
+      <c r="N1" s="47" t="n"/>
+      <c r="O1" s="47" t="n"/>
       <c r="P1" s="26" t="n"/>
       <c r="Q1" s="26" t="n"/>
       <c r="R1" s="29" t="inlineStr">
@@ -846,7 +892,7 @@
           <t>DATE / التاريخ</t>
         </is>
       </c>
-      <c r="S1" s="30" t="n"/>
+      <c r="S1" s="48" t="n"/>
       <c r="T1" s="31" t="inlineStr">
         <is>
           <t>….../….../.…</t>
@@ -857,18 +903,6 @@
       <c r="A2" s="32" t="n"/>
       <c r="B2" s="33" t="n"/>
       <c r="C2" s="33" t="n"/>
-      <c r="D2" s="33" t="n"/>
-      <c r="E2" s="33" t="n"/>
-      <c r="F2" s="33" t="n"/>
-      <c r="G2" s="33" t="n"/>
-      <c r="H2" s="33" t="n"/>
-      <c r="I2" s="33" t="n"/>
-      <c r="J2" s="33" t="n"/>
-      <c r="K2" s="33" t="n"/>
-      <c r="L2" s="33" t="n"/>
-      <c r="M2" s="33" t="n"/>
-      <c r="N2" s="33" t="n"/>
-      <c r="O2" s="33" t="n"/>
       <c r="P2" s="33" t="n"/>
       <c r="Q2" s="33" t="n"/>
       <c r="R2" s="29" t="inlineStr">
@@ -876,7 +910,7 @@
           <t>FORM NUMBER / رقم النموذج</t>
         </is>
       </c>
-      <c r="S2" s="30" t="n"/>
+      <c r="S2" s="48" t="n"/>
       <c r="T2" s="34" t="inlineStr">
         <is>
           <t>EMS.OR.FRM.21.01</t>
@@ -887,18 +921,6 @@
       <c r="A3" s="32" t="n"/>
       <c r="B3" s="33" t="n"/>
       <c r="C3" s="33" t="n"/>
-      <c r="D3" s="33" t="n"/>
-      <c r="E3" s="33" t="n"/>
-      <c r="F3" s="33" t="n"/>
-      <c r="G3" s="33" t="n"/>
-      <c r="H3" s="33" t="n"/>
-      <c r="I3" s="33" t="n"/>
-      <c r="J3" s="33" t="n"/>
-      <c r="K3" s="33" t="n"/>
-      <c r="L3" s="33" t="n"/>
-      <c r="M3" s="33" t="n"/>
-      <c r="N3" s="33" t="n"/>
-      <c r="O3" s="33" t="n"/>
       <c r="P3" s="33" t="n"/>
       <c r="Q3" s="33" t="n"/>
       <c r="R3" s="29" t="inlineStr">
@@ -906,7 +928,7 @@
           <t>REVISION / المراجعة</t>
         </is>
       </c>
-      <c r="S3" s="30" t="n"/>
+      <c r="S3" s="48" t="n"/>
       <c r="T3" s="31" t="inlineStr">
         <is>
           <t>R00</t>
@@ -917,18 +939,6 @@
       <c r="A4" s="32" t="n"/>
       <c r="B4" s="33" t="n"/>
       <c r="C4" s="33" t="n"/>
-      <c r="D4" s="33" t="n"/>
-      <c r="E4" s="33" t="n"/>
-      <c r="F4" s="33" t="n"/>
-      <c r="G4" s="33" t="n"/>
-      <c r="H4" s="33" t="n"/>
-      <c r="I4" s="33" t="n"/>
-      <c r="J4" s="33" t="n"/>
-      <c r="K4" s="33" t="n"/>
-      <c r="L4" s="33" t="n"/>
-      <c r="M4" s="33" t="n"/>
-      <c r="N4" s="33" t="n"/>
-      <c r="O4" s="33" t="n"/>
       <c r="P4" s="33" t="n"/>
       <c r="Q4" s="33" t="n"/>
       <c r="R4" s="29" t="inlineStr">
@@ -936,14 +946,13 @@
           <t>PUBLIC. DATE / تاريخ النشر</t>
         </is>
       </c>
-      <c r="S4" s="30" t="n"/>
+      <c r="S4" s="48" t="n"/>
       <c r="T4" s="31" t="inlineStr">
         <is>
           <t>19.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
         <is>
@@ -1049,7 +1058,6 @@
       <c r="S8" s="36" t="n"/>
       <c r="T8" s="37" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
         <is>
@@ -1382,7 +1390,6 @@
       <c r="S21" s="17" t="n"/>
       <c r="T21" s="37" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="35" t="inlineStr">
         <is>
@@ -1741,7 +1748,6 @@
       </c>
       <c r="T31" s="37" t="n"/>
     </row>
-    <row r="32"/>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="35" t="inlineStr">
         <is>
@@ -1820,40 +1826,39 @@
       <c r="S36" s="41" t="n"/>
       <c r="T36" s="11" t="n"/>
     </row>
-    <row r="37"/>
     <row r="38" ht="26" customHeight="1">
       <c r="A38" s="42" t="inlineStr">
         <is>
           <t>Warehouse / المستودع</t>
         </is>
       </c>
-      <c r="B38" s="43" t="n"/>
-      <c r="C38" s="43" t="n"/>
-      <c r="D38" s="43" t="n"/>
-      <c r="E38" s="43" t="n"/>
-      <c r="F38" s="43" t="n"/>
-      <c r="G38" s="44" t="n"/>
+      <c r="B38" s="36" t="n"/>
+      <c r="C38" s="36" t="n"/>
+      <c r="D38" s="36" t="n"/>
+      <c r="E38" s="36" t="n"/>
+      <c r="F38" s="36" t="n"/>
+      <c r="G38" s="37" t="n"/>
       <c r="H38" s="42" t="inlineStr">
         <is>
           <t>OCS / GOTS Coordinator / منسق OCS / GOTS</t>
         </is>
       </c>
-      <c r="I38" s="43" t="n"/>
-      <c r="J38" s="43" t="n"/>
-      <c r="K38" s="43" t="n"/>
-      <c r="L38" s="43" t="n"/>
-      <c r="M38" s="43" t="n"/>
-      <c r="N38" s="44" t="n"/>
+      <c r="I38" s="36" t="n"/>
+      <c r="J38" s="36" t="n"/>
+      <c r="K38" s="36" t="n"/>
+      <c r="L38" s="36" t="n"/>
+      <c r="M38" s="36" t="n"/>
+      <c r="N38" s="37" t="n"/>
       <c r="O38" s="42" t="inlineStr">
         <is>
           <t>Quality / الجودة</t>
         </is>
       </c>
-      <c r="P38" s="43" t="n"/>
-      <c r="Q38" s="43" t="n"/>
-      <c r="R38" s="43" t="n"/>
-      <c r="S38" s="43" t="n"/>
-      <c r="T38" s="44" t="n"/>
+      <c r="P38" s="36" t="n"/>
+      <c r="Q38" s="36" t="n"/>
+      <c r="R38" s="36" t="n"/>
+      <c r="S38" s="36" t="n"/>
+      <c r="T38" s="37" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="23" t="inlineStr">
@@ -1919,32 +1924,31 @@
       <c r="S41" s="41" t="n"/>
       <c r="T41" s="11" t="n"/>
     </row>
-    <row r="42"/>
     <row r="43" ht="32" customHeight="1">
       <c r="A43" s="35" t="inlineStr">
         <is>
           <t>Retention: at least 5 years or per certification body / customer requirement. Any nonconformity opens a corrective action (DÖF). | الاحتفاظ: 5 سنوات على الأقل أو حسب متطلبات جهة الاعتماد / العميل. وتفتح أي حالة عدم مطابقة إجراءً تصحيحيًا (DÖF).</t>
         </is>
       </c>
-      <c r="B43" s="43" t="n"/>
-      <c r="C43" s="43" t="n"/>
-      <c r="D43" s="43" t="n"/>
-      <c r="E43" s="43" t="n"/>
-      <c r="F43" s="43" t="n"/>
-      <c r="G43" s="43" t="n"/>
-      <c r="H43" s="43" t="n"/>
-      <c r="I43" s="43" t="n"/>
-      <c r="J43" s="43" t="n"/>
-      <c r="K43" s="43" t="n"/>
-      <c r="L43" s="43" t="n"/>
-      <c r="M43" s="43" t="n"/>
-      <c r="N43" s="43" t="n"/>
-      <c r="O43" s="43" t="n"/>
-      <c r="P43" s="43" t="n"/>
-      <c r="Q43" s="43" t="n"/>
-      <c r="R43" s="43" t="n"/>
-      <c r="S43" s="43" t="n"/>
-      <c r="T43" s="44" t="n"/>
+      <c r="B43" s="36" t="n"/>
+      <c r="C43" s="36" t="n"/>
+      <c r="D43" s="36" t="n"/>
+      <c r="E43" s="36" t="n"/>
+      <c r="F43" s="36" t="n"/>
+      <c r="G43" s="36" t="n"/>
+      <c r="H43" s="36" t="n"/>
+      <c r="I43" s="36" t="n"/>
+      <c r="J43" s="36" t="n"/>
+      <c r="K43" s="36" t="n"/>
+      <c r="L43" s="36" t="n"/>
+      <c r="M43" s="36" t="n"/>
+      <c r="N43" s="36" t="n"/>
+      <c r="O43" s="36" t="n"/>
+      <c r="P43" s="36" t="n"/>
+      <c r="Q43" s="36" t="n"/>
+      <c r="R43" s="36" t="n"/>
+      <c r="S43" s="36" t="n"/>
+      <c r="T43" s="37" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="145">

</xml_diff>